<commit_message>
90th Commit: Store_Text Keyword Implemted to Fetch data from locators
</commit_message>
<xml_diff>
--- a/APPLICATION1.xlsx
+++ b/APPLICATION1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vijay\Downloads\eit-automation-master\eit-automation-master\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E684600B-B3B1-4D40-A98B-95D21BFA9D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9FD566F-6AD1-4C9B-B28D-65E2F757F7BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SETUP" sheetId="1" r:id="rId1"/>
@@ -3498,18 +3498,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AMJ46"/>
-  <sheetFormatPr defaultRowHeight="13.9" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="13.95" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" style="1"/>
-    <col min="2" max="2" width="27.42578125" style="1"/>
-    <col min="3" max="3" width="24.42578125" style="1"/>
-    <col min="4" max="4" width="46.85546875" style="2"/>
-    <col min="5" max="5" width="83.42578125" style="3"/>
+    <col min="1" max="1" width="20.296875" style="1"/>
+    <col min="2" max="2" width="27.3984375" style="1"/>
+    <col min="3" max="3" width="24.3984375" style="1"/>
+    <col min="4" max="4" width="46.8984375" style="2"/>
+    <col min="5" max="5" width="83.3984375" style="3"/>
     <col min="6" max="6" width="69" style="3"/>
-    <col min="7" max="1024" width="13.140625" style="3"/>
+    <col min="7" max="1024" width="13.09765625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="3" customFormat="1" ht="12.75">
+    <row r="1" spans="1:6" s="3" customFormat="1" ht="13.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -3529,7 +3529,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="3" customFormat="1" ht="12.75">
+    <row r="2" spans="1:6" s="3" customFormat="1" ht="13.2">
       <c r="A2" s="2"/>
       <c r="B2" s="1" t="s">
         <v>6</v>
@@ -3556,7 +3556,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="4" spans="1:6" s="3" customFormat="1" ht="409.15" customHeight="1">
+    <row r="4" spans="1:6" s="3" customFormat="1" ht="409.2" customHeight="1">
       <c r="A4" s="2"/>
       <c r="B4" s="1" t="s">
         <v>11</v>
@@ -3586,7 +3586,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="6" spans="1:6" s="3" customFormat="1" ht="409.5">
+    <row r="6" spans="1:6" s="3" customFormat="1" ht="409.2">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
         <v>17</v>
@@ -3604,7 +3604,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="409.5">
+    <row r="7" spans="1:6" ht="409.6">
       <c r="B7" s="1" t="s">
         <v>20</v>
       </c>
@@ -3618,7 +3618,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="280.5">
+    <row r="8" spans="1:6" ht="290.39999999999998">
       <c r="B8" s="1" t="s">
         <v>23</v>
       </c>
@@ -3632,7 +3632,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="306">
+    <row r="9" spans="1:6" ht="316.8">
       <c r="B9" s="1" t="s">
         <v>26</v>
       </c>
@@ -3646,71 +3646,71 @@
         <v>277</v>
       </c>
     </row>
-    <row r="30" spans="4:5" ht="12.75">
+    <row r="30" spans="4:5" ht="13.2">
       <c r="D30" s="8"/>
       <c r="E30" s="8"/>
     </row>
-    <row r="31" spans="4:5" ht="12.75">
+    <row r="31" spans="4:5" ht="13.2">
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
     </row>
-    <row r="32" spans="4:5" ht="12.75">
+    <row r="32" spans="4:5" ht="13.2">
       <c r="D32" s="9"/>
       <c r="E32" s="9"/>
     </row>
-    <row r="33" spans="4:5" ht="12.75">
+    <row r="33" spans="4:5" ht="13.2">
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
     </row>
-    <row r="34" spans="4:5" ht="12.75">
+    <row r="34" spans="4:5" ht="13.2">
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
     </row>
-    <row r="35" spans="4:5" ht="12.75">
+    <row r="35" spans="4:5" ht="13.2">
       <c r="D35" s="9"/>
       <c r="E35" s="9"/>
     </row>
-    <row r="36" spans="4:5" ht="12.75">
+    <row r="36" spans="4:5" ht="13.2">
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
     </row>
-    <row r="37" spans="4:5" ht="12.75">
+    <row r="37" spans="4:5" ht="13.2">
       <c r="D37" s="9"/>
       <c r="E37" s="9"/>
     </row>
-    <row r="38" spans="4:5" ht="12.75">
+    <row r="38" spans="4:5" ht="13.2">
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
     </row>
-    <row r="39" spans="4:5" ht="12.75">
+    <row r="39" spans="4:5" ht="13.2">
       <c r="D39" s="9"/>
       <c r="E39" s="9"/>
     </row>
-    <row r="40" spans="4:5" ht="12.75">
+    <row r="40" spans="4:5" ht="13.2">
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
     </row>
-    <row r="41" spans="4:5" ht="12.75">
+    <row r="41" spans="4:5" ht="13.2">
       <c r="D41" s="9"/>
       <c r="E41" s="9"/>
     </row>
-    <row r="42" spans="4:5" ht="12.75">
+    <row r="42" spans="4:5" ht="13.2">
       <c r="D42" s="9"/>
       <c r="E42" s="9"/>
     </row>
-    <row r="43" spans="4:5" ht="12.75">
+    <row r="43" spans="4:5" ht="13.2">
       <c r="D43" s="9"/>
       <c r="E43" s="9"/>
     </row>
-    <row r="44" spans="4:5" ht="12.75">
+    <row r="44" spans="4:5" ht="13.2">
       <c r="D44" s="9"/>
       <c r="E44" s="9"/>
     </row>
-    <row r="45" spans="4:5" ht="12.75">
+    <row r="45" spans="4:5" ht="13.2">
       <c r="D45" s="9"/>
       <c r="E45" s="9"/>
     </row>
-    <row r="46" spans="4:5" ht="12.75">
+    <row r="46" spans="4:5" ht="13.2">
       <c r="D46" s="9"/>
       <c r="E46" s="9"/>
     </row>
@@ -3725,9 +3725,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.9" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="13.95" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="13.140625"/>
+    <col min="1" max="1" width="13.09765625"/>
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3737,9 +3737,9 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.9" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="13.95" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="13.140625"/>
+    <col min="1" max="1" width="13.09765625"/>
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3749,20 +3749,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AMJ49"/>
-  <sheetFormatPr defaultRowHeight="13.9" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="13.95" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="12.140625" style="2"/>
-    <col min="2" max="2" width="29.85546875" style="2"/>
-    <col min="3" max="3" width="28.42578125" style="2"/>
-    <col min="4" max="4" width="55.140625" style="2"/>
+    <col min="1" max="1" width="12.09765625" style="2"/>
+    <col min="2" max="2" width="29.8984375" style="2"/>
+    <col min="3" max="3" width="28.3984375" style="2"/>
+    <col min="4" max="4" width="55.09765625" style="2"/>
     <col min="5" max="5" width="87" style="3"/>
     <col min="6" max="6" width="265" style="3"/>
-    <col min="7" max="7" width="259.140625" style="3"/>
+    <col min="7" max="7" width="259.09765625" style="3"/>
     <col min="8" max="8" width="265" style="3"/>
-    <col min="9" max="1024" width="13.140625" style="3"/>
+    <col min="9" max="1024" width="13.09765625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="3" customFormat="1" ht="25.5">
+    <row r="1" spans="1:6" s="3" customFormat="1" ht="26.4">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -3799,7 +3799,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="357">
+    <row r="3" spans="1:6" ht="356.4">
       <c r="B3" s="1" t="s">
         <v>33</v>
       </c>
@@ -3810,7 +3810,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="140.25">
+    <row r="4" spans="1:6" ht="145.19999999999999">
       <c r="B4" s="1" t="s">
         <v>35</v>
       </c>
@@ -3824,7 +3824,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="306">
+    <row r="5" spans="1:6" ht="290.39999999999998">
       <c r="B5" s="1" t="s">
         <v>39</v>
       </c>
@@ -3838,7 +3838,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="306">
+    <row r="6" spans="1:6" ht="290.39999999999998">
       <c r="B6" s="1" t="s">
         <v>43</v>
       </c>
@@ -3852,7 +3852,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="306">
+    <row r="7" spans="1:6" ht="290.39999999999998">
       <c r="B7" s="1" t="s">
         <v>47</v>
       </c>
@@ -3866,7 +3866,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="293.25">
+    <row r="8" spans="1:6" ht="290.39999999999998">
       <c r="B8" s="1" t="s">
         <v>51</v>
       </c>
@@ -3880,7 +3880,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="306">
+    <row r="9" spans="1:6" ht="303.60000000000002">
       <c r="B9" s="1" t="s">
         <v>55</v>
       </c>
@@ -3894,7 +3894,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="369.75">
+    <row r="10" spans="1:6" ht="330">
       <c r="B10" s="1" t="s">
         <v>59</v>
       </c>
@@ -3908,7 +3908,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="318.75">
+    <row r="11" spans="1:6" ht="303.60000000000002">
       <c r="B11" s="1" t="s">
         <v>63</v>
       </c>
@@ -3922,7 +3922,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="280.5">
+    <row r="12" spans="1:6" ht="277.2">
       <c r="B12" s="1" t="s">
         <v>67</v>
       </c>
@@ -3936,7 +3936,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="408">
+    <row r="13" spans="1:6" ht="382.8">
       <c r="B13" s="1" t="s">
         <v>71</v>
       </c>
@@ -3950,7 +3950,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="318.75">
+    <row r="14" spans="1:6" ht="303.60000000000002">
       <c r="B14" s="1" t="s">
         <v>75</v>
       </c>
@@ -3964,7 +3964,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="331.5">
+    <row r="15" spans="1:6" ht="316.8">
       <c r="B15" s="1" t="s">
         <v>79</v>
       </c>
@@ -3978,7 +3978,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="331.5">
+    <row r="16" spans="1:6" ht="316.8">
       <c r="B16" s="1" t="s">
         <v>83</v>
       </c>
@@ -3992,7 +3992,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="63.75">
+    <row r="17" spans="1:8" ht="52.8">
       <c r="B17" s="1" t="s">
         <v>87</v>
       </c>
@@ -4006,7 +4006,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="242.25">
+    <row r="18" spans="1:8" ht="250.8">
       <c r="B18" s="1" t="s">
         <v>87</v>
       </c>
@@ -4020,7 +4020,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="76.5">
+    <row r="19" spans="1:8" ht="79.2">
       <c r="A19" s="1"/>
       <c r="B19" s="1" t="s">
         <v>87</v>
@@ -4038,7 +4038,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="102">
+    <row r="20" spans="1:8" ht="105.6">
       <c r="B20" s="1" t="s">
         <v>87</v>
       </c>
@@ -4055,7 +4055,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="76.5">
+    <row r="21" spans="1:8" ht="79.2">
       <c r="B21" s="1" t="s">
         <v>87</v>
       </c>
@@ -4086,7 +4086,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="23" spans="1:8" s="3" customFormat="1" ht="409.5">
+    <row r="23" spans="1:8" s="3" customFormat="1" ht="409.6">
       <c r="B23" s="1" t="s">
         <v>87</v>
       </c>
@@ -4109,7 +4109,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="191.25">
+    <row r="24" spans="1:8" ht="184.8">
       <c r="B24" s="1" t="s">
         <v>115</v>
       </c>
@@ -4141,7 +4141,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="26" spans="1:8" s="12" customFormat="1" ht="409.5">
+    <row r="26" spans="1:8" s="12" customFormat="1" ht="409.6">
       <c r="A26" s="11"/>
       <c r="B26" s="11" t="s">
         <v>124</v>
@@ -4156,7 +4156,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="27" spans="1:8" s="3" customFormat="1" ht="409.5">
+    <row r="27" spans="1:8" s="3" customFormat="1" ht="409.6">
       <c r="A27" s="2"/>
       <c r="B27" s="2" t="s">
         <v>128</v>
@@ -4174,7 +4174,7 @@
       <c r="G27" s="9"/>
       <c r="H27" s="9"/>
     </row>
-    <row r="28" spans="1:8" s="3" customFormat="1" ht="409.5">
+    <row r="28" spans="1:8" s="3" customFormat="1" ht="409.6">
       <c r="B28" s="2" t="s">
         <v>132</v>
       </c>
@@ -4191,7 +4191,7 @@
       <c r="G28" s="9"/>
       <c r="H28" s="9"/>
     </row>
-    <row r="29" spans="1:8" s="3" customFormat="1" ht="408">
+    <row r="29" spans="1:8" s="3" customFormat="1" ht="409.6">
       <c r="B29" s="2" t="s">
         <v>136</v>
       </c>
@@ -4208,7 +4208,7 @@
       <c r="G29" s="9"/>
       <c r="H29" s="9"/>
     </row>
-    <row r="30" spans="1:8" s="3" customFormat="1" ht="395.25">
+    <row r="30" spans="1:8" s="3" customFormat="1" ht="409.2">
       <c r="B30" s="15" t="s">
         <v>140</v>
       </c>
@@ -4225,7 +4225,7 @@
       <c r="G30" s="9"/>
       <c r="H30" s="9"/>
     </row>
-    <row r="31" spans="1:8" s="3" customFormat="1" ht="331.5">
+    <row r="31" spans="1:8" s="3" customFormat="1" ht="343.2">
       <c r="B31" s="2" t="s">
         <v>144</v>
       </c>
@@ -4242,7 +4242,7 @@
       <c r="G31" s="9"/>
       <c r="H31" s="9"/>
     </row>
-    <row r="32" spans="1:8" s="3" customFormat="1" ht="395.25">
+    <row r="32" spans="1:8" s="3" customFormat="1" ht="382.8">
       <c r="B32" s="14" t="s">
         <v>148</v>
       </c>
@@ -4259,7 +4259,7 @@
       <c r="G32" s="9"/>
       <c r="H32" s="9"/>
     </row>
-    <row r="33" spans="2:8" s="3" customFormat="1" ht="409.5">
+    <row r="33" spans="2:8" s="3" customFormat="1" ht="409.6">
       <c r="B33" s="14" t="s">
         <v>152</v>
       </c>
@@ -4276,7 +4276,7 @@
       <c r="G33" s="9"/>
       <c r="H33" s="9"/>
     </row>
-    <row r="34" spans="2:8" s="3" customFormat="1" ht="267.75">
+    <row r="34" spans="2:8" s="3" customFormat="1" ht="277.2">
       <c r="B34" s="7" t="s">
         <v>156</v>
       </c>
@@ -4293,7 +4293,7 @@
       <c r="G34" s="9"/>
       <c r="H34" s="9"/>
     </row>
-    <row r="35" spans="2:8" s="3" customFormat="1" ht="293.25">
+    <row r="35" spans="2:8" s="3" customFormat="1" ht="303.60000000000002">
       <c r="B35" s="7" t="s">
         <v>160</v>
       </c>
@@ -4310,7 +4310,7 @@
       <c r="G35" s="9"/>
       <c r="H35" s="9"/>
     </row>
-    <row r="36" spans="2:8" s="3" customFormat="1" ht="409.5">
+    <row r="36" spans="2:8" s="3" customFormat="1" ht="409.6">
       <c r="B36" s="7" t="s">
         <v>164</v>
       </c>
@@ -4327,7 +4327,7 @@
       <c r="G36" s="9"/>
       <c r="H36" s="9"/>
     </row>
-    <row r="37" spans="2:8" s="3" customFormat="1" ht="409.5">
+    <row r="37" spans="2:8" s="3" customFormat="1" ht="409.6">
       <c r="B37" s="7" t="s">
         <v>168</v>
       </c>
@@ -4344,7 +4344,7 @@
       <c r="G37" s="9"/>
       <c r="H37" s="9"/>
     </row>
-    <row r="38" spans="2:8" s="3" customFormat="1" ht="408">
+    <row r="38" spans="2:8" s="3" customFormat="1" ht="409.6">
       <c r="B38" s="7" t="s">
         <v>172</v>
       </c>
@@ -4361,7 +4361,7 @@
       <c r="G38" s="9"/>
       <c r="H38" s="9"/>
     </row>
-    <row r="39" spans="2:8" s="3" customFormat="1" ht="318.75">
+    <row r="39" spans="2:8" s="3" customFormat="1" ht="330">
       <c r="B39" s="7" t="s">
         <v>176</v>
       </c>
@@ -4378,7 +4378,7 @@
       <c r="G39" s="9"/>
       <c r="H39" s="9"/>
     </row>
-    <row r="40" spans="2:8" s="3" customFormat="1" ht="409.5">
+    <row r="40" spans="2:8" s="3" customFormat="1" ht="409.6">
       <c r="B40" s="7" t="s">
         <v>180</v>
       </c>
@@ -4395,7 +4395,7 @@
       <c r="G40" s="9"/>
       <c r="H40" s="9"/>
     </row>
-    <row r="41" spans="2:8" s="3" customFormat="1" ht="409.5">
+    <row r="41" spans="2:8" s="3" customFormat="1" ht="409.6">
       <c r="B41" s="7" t="s">
         <v>184</v>
       </c>
@@ -4412,7 +4412,7 @@
       <c r="G41" s="9"/>
       <c r="H41" s="9"/>
     </row>
-    <row r="42" spans="2:8" s="3" customFormat="1" ht="369.75">
+    <row r="42" spans="2:8" s="3" customFormat="1" ht="382.8">
       <c r="B42" s="15" t="s">
         <v>188</v>
       </c>
@@ -4429,7 +4429,7 @@
       <c r="G42" s="9"/>
       <c r="H42" s="9"/>
     </row>
-    <row r="43" spans="2:8" s="3" customFormat="1" ht="409.5">
+    <row r="43" spans="2:8" s="3" customFormat="1" ht="396">
       <c r="B43" s="2" t="s">
         <v>192</v>
       </c>
@@ -4446,7 +4446,7 @@
       <c r="G43" s="9"/>
       <c r="H43" s="9"/>
     </row>
-    <row r="44" spans="2:8" s="3" customFormat="1" ht="293.25">
+    <row r="44" spans="2:8" s="3" customFormat="1" ht="290.39999999999998">
       <c r="B44" s="2" t="s">
         <v>196</v>
       </c>
@@ -4463,7 +4463,7 @@
       <c r="G44" s="9"/>
       <c r="H44" s="9"/>
     </row>
-    <row r="45" spans="2:8" ht="318.75">
+    <row r="45" spans="2:8" ht="330">
       <c r="B45" s="2" t="s">
         <v>200</v>
       </c>
@@ -4477,7 +4477,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="46" spans="2:8" ht="255">
+    <row r="46" spans="2:8" ht="264">
       <c r="B46" s="2" t="s">
         <v>204</v>
       </c>
@@ -4491,7 +4491,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="47" spans="2:8" ht="409.5">
+    <row r="47" spans="2:8" ht="409.6">
       <c r="B47" s="2" t="s">
         <v>208</v>
       </c>
@@ -4505,7 +4505,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="48" spans="2:8" ht="255">
+    <row r="48" spans="2:8" ht="224.4">
       <c r="B48" s="2" t="s">
         <v>212</v>
       </c>
@@ -4519,7 +4519,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="49" spans="2:5" ht="102">
+    <row r="49" spans="2:5" ht="92.4">
       <c r="B49" s="2" t="s">
         <v>216</v>
       </c>
@@ -4556,17 +4556,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F27"/>
-  <sheetFormatPr defaultRowHeight="13.9" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="13.95" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="22.140625"/>
-    <col min="2" max="3" width="35.42578125"/>
-    <col min="4" max="4" width="46.42578125"/>
-    <col min="5" max="5" width="65.28515625"/>
-    <col min="6" max="6" width="72.42578125"/>
-    <col min="7" max="1024" width="13.140625"/>
+    <col min="1" max="1" width="22.09765625"/>
+    <col min="2" max="3" width="35.3984375"/>
+    <col min="4" max="4" width="46.3984375"/>
+    <col min="5" max="5" width="65.296875"/>
+    <col min="6" max="6" width="72.3984375"/>
+    <col min="7" max="1024" width="13.09765625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="3" customFormat="1" ht="12.75">
+    <row r="1" spans="1:6" s="3" customFormat="1" ht="13.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -4603,7 +4603,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="3" spans="1:6" s="3" customFormat="1" ht="409.5">
+    <row r="3" spans="1:6" s="3" customFormat="1" ht="409.6">
       <c r="A3" s="2"/>
       <c r="B3" s="1" t="s">
         <v>33</v>
@@ -4618,7 +4618,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="4" spans="1:6" s="3" customFormat="1" ht="140.25">
+    <row r="4" spans="1:6" s="3" customFormat="1" ht="145.19999999999999">
       <c r="A4" s="2"/>
       <c r="B4" s="1" t="s">
         <v>35</v>
@@ -4633,7 +4633,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:6" s="3" customFormat="1" ht="409.5">
+    <row r="5" spans="1:6" s="3" customFormat="1" ht="409.6">
       <c r="A5" s="2"/>
       <c r="B5" s="1" t="s">
         <v>224</v>
@@ -4648,7 +4648,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="6" spans="1:6" s="3" customFormat="1" ht="409.5">
+    <row r="6" spans="1:6" s="3" customFormat="1" ht="409.6">
       <c r="A6" s="2"/>
       <c r="B6" s="1" t="s">
         <v>228</v>
@@ -4663,7 +4663,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="7" spans="1:6" s="3" customFormat="1" ht="409.5">
+    <row r="7" spans="1:6" s="3" customFormat="1" ht="409.6">
       <c r="A7" s="2"/>
       <c r="B7" s="1" t="s">
         <v>232</v>
@@ -4678,7 +4678,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="8" spans="1:6" s="3" customFormat="1" ht="409.5">
+    <row r="8" spans="1:6" s="3" customFormat="1" ht="409.6">
       <c r="A8" s="2"/>
       <c r="B8" s="1" t="s">
         <v>236</v>
@@ -4693,7 +4693,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="9" spans="1:6" s="3" customFormat="1" ht="409.5">
+    <row r="9" spans="1:6" s="3" customFormat="1" ht="409.6">
       <c r="A9" s="2"/>
       <c r="B9" s="1" t="s">
         <v>240</v>
@@ -4708,7 +4708,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="10" spans="1:6" s="3" customFormat="1" ht="102">
+    <row r="10" spans="1:6" s="3" customFormat="1" ht="105.6">
       <c r="A10" s="2"/>
       <c r="B10" s="1" t="s">
         <v>87</v>
@@ -4723,7 +4723,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="11" spans="1:6" s="3" customFormat="1" ht="127.5">
+    <row r="11" spans="1:6" s="3" customFormat="1" ht="132">
       <c r="A11" s="2"/>
       <c r="B11" s="1" t="s">
         <v>87</v>
@@ -4738,7 +4738,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="12" spans="1:6" s="3" customFormat="1" ht="63.75">
+    <row r="12" spans="1:6" s="3" customFormat="1" ht="66">
       <c r="A12" s="1"/>
       <c r="B12" s="1" t="s">
         <v>87</v>
@@ -4753,7 +4753,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="13" spans="1:6" s="3" customFormat="1" ht="63.75">
+    <row r="13" spans="1:6" s="3" customFormat="1" ht="66">
       <c r="A13" s="2"/>
       <c r="B13" s="1" t="s">
         <v>87</v>
@@ -4768,7 +4768,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="14" spans="1:6" s="3" customFormat="1" ht="63.75">
+    <row r="14" spans="1:6" s="3" customFormat="1" ht="66">
       <c r="A14" s="2"/>
       <c r="B14" s="1" t="s">
         <v>87</v>
@@ -4783,7 +4783,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="15" spans="1:6" s="3" customFormat="1" ht="73.150000000000006" customHeight="1">
+    <row r="15" spans="1:6" s="3" customFormat="1" ht="73.2" customHeight="1">
       <c r="A15" s="2"/>
       <c r="B15" s="1" t="s">
         <v>87</v>
@@ -4798,7 +4798,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="16" spans="1:6" s="3" customFormat="1" ht="63.75">
+    <row r="16" spans="1:6" s="3" customFormat="1" ht="66">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
         <v>87</v>
@@ -4813,7 +4813,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="17" spans="1:5" s="3" customFormat="1" ht="63.75">
+    <row r="17" spans="1:5" s="3" customFormat="1" ht="66">
       <c r="A17" s="1"/>
       <c r="B17" s="1" t="s">
         <v>87</v>
@@ -4828,7 +4828,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="63.75">
+    <row r="18" spans="1:5" ht="66">
       <c r="B18" s="1" t="s">
         <v>87</v>
       </c>
@@ -4842,7 +4842,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="19" spans="1:5" s="18" customFormat="1" ht="63.75">
+    <row r="19" spans="1:5" s="18" customFormat="1" ht="66">
       <c r="B19" s="1" t="s">
         <v>87</v>
       </c>
@@ -4856,7 +4856,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="20" spans="1:5" s="18" customFormat="1" ht="63.75">
+    <row r="20" spans="1:5" s="18" customFormat="1" ht="66">
       <c r="B20" s="1" t="s">
         <v>87</v>
       </c>
@@ -4870,7 +4870,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="21" spans="1:5" s="3" customFormat="1" ht="127.5">
+    <row r="21" spans="1:5" s="3" customFormat="1" ht="132">
       <c r="A21" s="2"/>
       <c r="B21" s="1" t="s">
         <v>115</v>
@@ -4900,19 +4900,19 @@
         <v>268</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="12.75">
+    <row r="23" spans="1:5" ht="13.2">
       <c r="B23" s="18"/>
     </row>
-    <row r="24" spans="1:5" ht="12.75">
+    <row r="24" spans="1:5" ht="13.2">
       <c r="B24" s="18"/>
     </row>
-    <row r="25" spans="1:5" ht="12.75">
+    <row r="25" spans="1:5" ht="13.2">
       <c r="B25" s="18"/>
     </row>
-    <row r="26" spans="1:5" ht="12.75">
+    <row r="26" spans="1:5" ht="13.2">
       <c r="B26" s="18"/>
     </row>
-    <row r="27" spans="1:5" ht="12.75">
+    <row r="27" spans="1:5" ht="13.2">
       <c r="B27" s="18"/>
     </row>
   </sheetData>
@@ -4930,18 +4930,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="13.9" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="13.95" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="14.28515625"/>
-    <col min="2" max="2" width="18.7109375"/>
-    <col min="3" max="3" width="15.85546875"/>
-    <col min="4" max="4" width="44.42578125"/>
-    <col min="5" max="5" width="52.5703125"/>
-    <col min="6" max="6" width="20.28515625"/>
-    <col min="7" max="8" width="13.140625"/>
+    <col min="1" max="1" width="14.296875"/>
+    <col min="2" max="2" width="18.69921875"/>
+    <col min="3" max="3" width="15.8984375"/>
+    <col min="4" max="4" width="44.3984375"/>
+    <col min="5" max="5" width="52.59765625"/>
+    <col min="6" max="6" width="20.296875"/>
+    <col min="7" max="8" width="13.09765625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="13.9" customHeight="1">
+    <row r="1" spans="1:8" ht="13.95" customHeight="1">
       <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
@@ -4963,11 +4963,11 @@
       <c r="G1" s="21"/>
       <c r="H1" s="21"/>
     </row>
-    <row r="2" spans="1:8" ht="13.9" customHeight="1">
+    <row r="2" spans="1:8" ht="13.95" customHeight="1">
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:8" ht="13.9" customHeight="1">
+    <row r="3" spans="1:8" ht="13.95" customHeight="1">
       <c r="A3" s="18"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
@@ -4980,12 +4980,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.9" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="13.95" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="13.140625"/>
+    <col min="1" max="1" width="13.09765625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="13.9" customHeight="1">
+    <row r="1" spans="1:1" ht="13.95" customHeight="1">
       <c r="A1" t="s">
         <v>269</v>
       </c>
@@ -4998,12 +4998,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.9" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="13.95" customHeight="1"/>
   <cols>
-    <col min="1" max="3" width="13.140625"/>
+    <col min="1" max="3" width="13.09765625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="13.9" customHeight="1">
+    <row r="1" spans="1:1" ht="13.95" customHeight="1">
       <c r="A1" t="s">
         <v>270</v>
       </c>
@@ -5016,17 +5016,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="13.9" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="13.95" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="13.140625"/>
-    <col min="2" max="2" width="24.140625"/>
-    <col min="3" max="3" width="16.28515625"/>
-    <col min="4" max="4" width="39.5703125"/>
-    <col min="5" max="5" width="63.28515625"/>
-    <col min="6" max="1024" width="13.140625"/>
+    <col min="1" max="1" width="13.09765625"/>
+    <col min="2" max="2" width="24.09765625"/>
+    <col min="3" max="3" width="16.296875"/>
+    <col min="4" max="4" width="39.59765625"/>
+    <col min="5" max="5" width="63.296875"/>
+    <col min="6" max="1024" width="13.09765625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="3" customFormat="1" ht="25.5">
+    <row r="1" spans="1:6" s="3" customFormat="1" ht="13.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -5046,7 +5046,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="3" customFormat="1" ht="153">
+    <row r="2" spans="1:6" s="3" customFormat="1" ht="158.4">
       <c r="A2" s="2" t="s">
         <v>29</v>
       </c>
@@ -5071,9 +5071,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.9" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="13.95" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="13.140625"/>
+    <col min="1" max="1" width="13.09765625"/>
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5083,9 +5083,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.9" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="13.95" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="13.140625"/>
+    <col min="1" max="1" width="13.09765625"/>
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>